<commit_message>
Hoan thanh chinh sua Data
</commit_message>
<xml_diff>
--- a/TestData/checkout_error.xlsx
+++ b/TestData/checkout_error.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Software Testing\TestData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Software Testing\TestSauceDemo\WebSauceDemo\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{166D8EDD-08B9-498B-97A9-DD903B9A2CB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95AE1EC0-6C26-4191-B9C6-F2C340B5B111}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3072" yWindow="4104" windowWidth="18420" windowHeight="10680" xr2:uid="{EA0A8AE1-9B76-405F-8047-5F61C03A2185}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="24792" windowHeight="14856" xr2:uid="{EA0A8AE1-9B76-405F-8047-5F61C03A2185}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -518,7 +518,7 @@
     <col min="1" max="1" width="11.21875" customWidth="1"/>
     <col min="2" max="2" width="11" customWidth="1"/>
     <col min="3" max="3" width="15.109375" customWidth="1"/>
-    <col min="4" max="4" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>